<commit_message>
Guia de formulas: cada formula como una pregunta simple y la cuenta en palabras de todos los dias (tambien en el Excel)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/descargas/10-formulas-financieras-restaurante.xlsx
+++ b/descargas/10-formulas-financieras-restaurante.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Qué te dice</t>
+          <t>Te responde</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -623,12 +623,12 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Lo que te queda de cada peso vendido después de pagar la mercadería.</t>
+          <t>¿Cuánto te queda después de la mercadería?</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>(Ventas − CMV) ÷ Ventas × 100</t>
+          <t>(Ventas − Mercadería) ÷ Ventas × 100</t>
         </is>
       </c>
       <c r="F6" s="8">
@@ -656,7 +656,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>(Precio − Costo variable) ÷ Precio × 100</t>
+          <t>(Precio − Lo que te cuesta hacerlo) ÷ Precio × 100</t>
         </is>
       </c>
       <c r="F7" s="8">
@@ -679,12 +679,12 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Lo que genera la operación, antes de intereses, impuestos y amortizaciones.</t>
+          <t>¿Cuánto gana el local con su trabajo, antes de intereses, impuestos y desgaste de equipos?</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Utilidad operativa + Amortizaciones</t>
+          <t>Ganancia del local + Desgaste de los equipos</t>
         </is>
       </c>
       <c r="F8" s="9">
@@ -712,7 +712,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Costos fijos ÷ Margen de contribución %</t>
+          <t>Gastos fijos ÷ Margen de todo el local</t>
         </is>
       </c>
       <c r="F9" s="9">
@@ -735,20 +735,20 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Si podés pagar las deudas de corto plazo sin vender mercadería.</t>
+          <t>¿Te alcanza para pagar lo que debés, sin contar la mercadería?</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>(Activo corriente − Inventario) ÷ Pasivo corriente</t>
+          <t>(Caja y banco + Lo que te deben) ÷ Lo que tenés que pagar este año</t>
         </is>
       </c>
       <c r="F10" s="10">
-        <f>IFERROR(('Tus números'!$C$18-'Tus números'!$C$19)/'Tus números'!$C$20,"")</f>
+        <f>IFERROR(('Tus números'!$C$18+'Tus números'!$C$19)/'Tus números'!$C$20,"")</f>
         <v/>
       </c>
       <c r="G10" s="6">
-        <f>IF(F10="","Cargá activo, inventario y pasivo.",IF(F10&gt;=1,"Mayor a 1: estás cubierto.","Menor a 1: hoy no te alcanza para pagar todo lo de corto plazo."))</f>
+        <f>IF(F10="","Cargá tu plata, lo que te deben y lo que debés.",IF(F10&gt;=1,"Más de 1: estás cubierto.","Menos de 1: hoy no te alcanza para pagar todo lo que vence este año."))</f>
         <v/>
       </c>
     </row>
@@ -758,12 +758,12 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Ciclo de conversión de efectivo</t>
+          <t>Ciclo de caja</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Cuántos días tarda la plata que ponés en volver a tu caja.</t>
+          <t>¿En cuántos días vuelve a la caja la plata que ponés en mercadería?</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -786,17 +786,17 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>ROI (retorno sobre la inversión)</t>
+          <t>ROI</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Cuánto rinde cada peso puesto en el negocio, contando lo prestado.</t>
+          <t>¿Cuánto rinde por año todo lo que se puso en el negocio?</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Ganancia neta anual ÷ Inversión total × 100</t>
+          <t>Ganancia del año ÷ Todo lo que se puso × 100</t>
         </is>
       </c>
       <c r="F12" s="8">
@@ -804,7 +804,7 @@
         <v/>
       </c>
       <c r="G12" s="6">
-        <f>IF(F12="","Cargá ganancia e inversión.","Recuperás la inversión en unos "&amp;ROUND(1/F12,1)&amp;" años. Comparalo con la tasa de la hoja ""Tus números"" ("&amp;TEXT('Tus números'!$C$31,"0%")&amp;").")</f>
+        <f>IF(F12="","Cargá la ganancia y lo que se puso.","Recuperás la inversión en unos "&amp;ROUND(1/F12,1)&amp;" años. Comparalo con la tasa de la hoja ""Tus números"" ("&amp;TEXT('Tus números'!$C$31,"0%")&amp;").")</f>
         <v/>
       </c>
     </row>
@@ -814,17 +814,17 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>ROE (retorno sobre el patrimonio)</t>
+          <t>ROE</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Cuánto rinde la plata que es tuya.</t>
+          <t>¿Cuánto rinde por año la plata que pusiste vos?</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Ganancia neta anual ÷ Patrimonio neto × 100</t>
+          <t>Ganancia del año ÷ Lo que pusiste vos × 100</t>
         </is>
       </c>
       <c r="F13" s="8">
@@ -832,7 +832,7 @@
         <v/>
       </c>
       <c r="G13" s="6">
-        <f>IF(F13="","Cargá ganancia y patrimonio.",IF(F13&gt;'Tus números'!$C$31,"Tu plata rinde más que la tasa de la hoja ""Tus números"" ("&amp;TEXT('Tus números'!$C$31,"0%")&amp;").","Tu plata rinde igual o menos que la tasa de la hoja ""Tus números"" ("&amp;TEXT('Tus números'!$C$31,"0%")&amp;"): en otro lado ganarías parecido."))</f>
+        <f>IF(F13="","Cargá la ganancia y lo que pusiste vos.",IF(F13&gt;'Tus números'!$C$31,"Tu plata rinde más que la tasa de la hoja ""Tus números"" ("&amp;TEXT('Tus números'!$C$31,"0%")&amp;").","Tu plata rinde igual o menos que la tasa de la hoja ""Tus números"" ("&amp;TEXT('Tus números'!$C$31,"0%")&amp;"): en otro lado ganarías parecido."))</f>
         <v/>
       </c>
     </row>
@@ -842,17 +842,17 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>VPN (valor presente neto)</t>
+          <t>VPN</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Cuánto vale hoy lo que una inversión te va a dar.</t>
+          <t>¿Te conviene esta inversión?</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Flujos futuros descontados − Inversión inicial</t>
+          <t>Lo que te deja, en plata de hoy − Lo que ponés</t>
         </is>
       </c>
       <c r="F14" s="9">
@@ -870,12 +870,12 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>TIR (tasa interna de retorno)</t>
+          <t>TIR</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>La rentabilidad de esa inversión, en % por año.</t>
+          <t>¿Cuánto te rinde por año esta inversión?</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -958,7 +958,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Costo de la mercadería vendida (CMV)</t>
+          <t>Mercadería vendida</t>
         </is>
       </c>
       <c r="C8" s="15" t="n">
@@ -966,14 +966,14 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>Lo que te costó la comida y la bebida que vendiste en el mes.</t>
+          <t>Lo que te costó la comida y la bebida que vendiste en el mes (tu contador le dice CMV).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>Otros costos variables</t>
+          <t>Envases y comisiones</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
@@ -988,7 +988,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Costos fijos del mes (sin amortizaciones)</t>
+          <t>Gastos fijos del mes (sin el desgaste de equipos)</t>
         </is>
       </c>
       <c r="C10" s="15" t="n">
@@ -1003,7 +1003,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Amortizaciones del mes</t>
+          <t>Desgaste de los equipos por mes</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>Lo que se gasta por mes de lo que compraste para usar años (horno, heladera, obra). Ej: horno de $12.000.000 que dura 10 años = $100.000 por mes.</t>
+          <t>Horno, heladera, obra: lo que pagaste dividido por los meses que dura. Ej: horno de $12.000.000 que dura 10 años = $100.000 por mes. Tu contador le dice amortizaciones.</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Costo variable de ese producto</t>
+          <t>Lo que te cuesta hacerlo</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
@@ -1055,29 +1055,29 @@
     <row r="17" ht="24" customHeight="1">
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Hoy (sacalo del balance o de tu contador)</t>
+          <t>Hoy</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Activo corriente</t>
+          <t>Plata en caja y banco</t>
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>12000000</v>
+        <v>6000000</v>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>Caja, banco, lo que te deben cobrar en menos de un año y la mercadería.</t>
+          <t>Lo que tenés hoy en efectivo y en el banco.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Inventario (mercadería en stock)</t>
+          <t>Lo que te deben</t>
         </is>
       </c>
       <c r="C19" s="15" t="n">
@@ -1085,14 +1085,14 @@
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>Lo que vale la mercadería que tenés hoy en depósito y cámaras.</t>
+          <t>Tarjetas y apps que todavía no te pagaron, clientes con cuenta.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Pasivo corriente</t>
+          <t>Lo que tenés que pagar este año</t>
         </is>
       </c>
       <c r="C20" s="15" t="n">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>Lo que tenés que pagar en menos de un año: proveedores, sueldos, impuestos, cuotas.</t>
+          <t>Proveedores, sueldos, impuestos y cuotas de préstamos que vencen en los próximos 12 meses.</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
     <row r="26" ht="30" customHeight="1">
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Ganancia neta del año</t>
+          <t>Ganancia del año</t>
         </is>
       </c>
       <c r="C26" s="15" t="n">
@@ -1167,14 +1167,14 @@
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>Lo que quedó después de todo: costos, intereses e impuestos.</t>
+          <t>Lo que quedó después de pagar todo: costos, intereses e impuestos.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Inversión total en el negocio</t>
+          <t>Todo lo que se puso en el negocio</t>
         </is>
       </c>
       <c r="C27" s="15" t="n">
@@ -1182,14 +1182,14 @@
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>Todo lo que se puso para armarlo y hacerlo andar: obra, equipos, mercadería y caja. Lo tuyo y lo prestado.</t>
+          <t>Obra, equipos, mercadería y caja para arrancar. Lo tuyo y lo prestado.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>Patrimonio neto (lo que es tuyo)</t>
+          <t>Lo que pusiste vos</t>
         </is>
       </c>
       <c r="C28" s="15" t="n">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>La inversión total menos lo que debés (préstamos).</t>
+          <t>Lo de arriba menos lo que pediste prestado.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Guia de formulas: el EBITDA pasa a llamarse lo que genera tu local
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/descargas/10-formulas-financieras-restaurante.xlsx
+++ b/descargas/10-formulas-financieras-restaurante.xlsx
@@ -674,12 +674,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>EBITDA</t>
+          <t>Lo que genera tu local (EBITDA)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>¿Cuánto gana el local con su trabajo, antes de intereses, impuestos y desgaste de equipos?</t>
+          <t>¿Cuánto genera el local con su trabajo, antes de intereses, impuestos y desgaste de equipos?</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Guia de formulas: el EBITDA se llama ganancia de la operacion
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/descargas/10-formulas-financieras-restaurante.xlsx
+++ b/descargas/10-formulas-financieras-restaurante.xlsx
@@ -674,17 +674,17 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Lo que genera tu local (EBITDA)</t>
+          <t>Ganancia de la operación (EBITDA)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>¿Cuánto genera el local con su trabajo, antes de intereses, impuestos y desgaste de equipos?</t>
+          <t>¿Cuánto gana el local con su trabajo, antes de intereses, impuestos y desgaste de equipos?</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Ganancia del local + Desgaste de los equipos</t>
+          <t>Lo que queda después de todos los gastos + Desgaste de los equipos</t>
         </is>
       </c>
       <c r="F8" s="9">

</xml_diff>